<commit_message>
updated Threat Prioritization - Candidate Ranking materials (spelling error in ranking template)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCDL threat candidate ranking template.xlsx
+++ b/distribution/reference_documents/templates/AVCDL threat candidate ranking template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C1EED1-3167-3F49-BF7B-E18C95A53F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A4A9AA-8BF7-8D47-9760-C5288828257C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-59940" yWindow="-31880" windowWidth="37960" windowHeight="22360" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
+    <workbookView xWindow="-73200" yWindow="-33080" windowWidth="37960" windowHeight="22360" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="7" r:id="rId1"/>
@@ -115,13 +115,7 @@
     <t>rubric value</t>
   </si>
   <si>
-    <t>rubric quantiazation</t>
-  </si>
-  <si>
     <t>candidate ID</t>
-  </si>
-  <si>
-    <t>domain quantiazation</t>
   </si>
   <si>
     <t>Domain Quantization</t>
@@ -247,6 +241,12 @@
   </si>
   <si>
     <t>Likelihood Rubric</t>
+  </si>
+  <si>
+    <t>rubric quantization</t>
+  </si>
+  <si>
+    <t>domain quantization</t>
   </si>
 </sst>
 </file>
@@ -555,6 +555,10 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -565,10 +569,6 @@
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -911,18 +911,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="59" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
+      <c r="B2" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="6"/>
@@ -941,15 +941,15 @@
         <v>13</v>
       </c>
       <c r="C4" s="48"/>
-      <c r="D4" s="54" t="s">
+      <c r="D4" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
       <c r="K4" s="6"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
@@ -966,18 +966,18 @@
     </row>
     <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.3">
       <c r="B6" s="47" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C6" s="48"/>
-      <c r="D6" s="54" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
+      <c r="D6" s="56" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
       <c r="K6" s="6"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
@@ -997,15 +997,15 @@
         <v>2</v>
       </c>
       <c r="C8" s="48"/>
-      <c r="D8" s="55">
+      <c r="D8" s="57">
         <v>36765</v>
       </c>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
-      <c r="J8" s="55"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="57"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="57"/>
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -1049,18 +1049,18 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:11" ht="23" x14ac:dyDescent="0.2">
-      <c r="B12" s="53" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="53"/>
-      <c r="J12" s="53"/>
-      <c r="K12" s="53"/>
+      <c r="B12" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1090,11 +1090,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1219,11 +1219,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1247,24 +1247,24 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="39" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" s="39" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -1356,23 +1356,22 @@
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="14.5" customWidth="1"/>
+    <col min="8" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
+      <c r="B2" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1391,28 +1390,28 @@
     <row r="4" spans="1:13" ht="49" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>12</v>
@@ -1779,17 +1778,17 @@
       <c r="J28" s="6"/>
     </row>
     <row r="29" spans="2:10" ht="20" x14ac:dyDescent="0.2">
-      <c r="B29" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" s="57"/>
-      <c r="D29" s="57"/>
-      <c r="E29" s="57"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
+      <c r="B29" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="53"/>
+      <c r="D29" s="53"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="53"/>
+      <c r="G29" s="53"/>
+      <c r="H29" s="53"/>
+      <c r="I29" s="53"/>
+      <c r="J29" s="53"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
@@ -1966,12 +1965,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -2123,12 +2122,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="56" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
+      <c r="B2" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -2400,7 +2399,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="9"/>

</xml_diff>